<commit_message>
Add Arabic names and missing information to member data
Update `test_members_150_EN.xlsx` with Arabic names and missing emails, and add 2026 subscriptions to `test_subscriptions_EN.xlsx`.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 9ac71dc7-50b4-4cca-8443-0dbf64795da8
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: e520eed1-2cda-4121-98ea-73b89f96cc21
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/014c195b-b384-40b2-b0f0-f245ec252029/9ac71dc7-50b4-4cca-8443-0dbf64795da8/glPN9Jq
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/ملفات_للتحميل/test_members_150_EN.xlsx
+++ b/ملفات_للتحميل/test_members_150_EN.xlsx
@@ -398,23 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O151"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="13.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="21.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="14.83203125" customWidth="1"/>
-    <col min="13" max="13" width="12.83203125" customWidth="1"/>
-    <col min="14" max="14" width="17.83203125" customWidth="1"/>
-    <col min="15" max="15" width="12.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -471,7 +454,7 @@
         <v>Bakri</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>صالح طارق بكري</v>
       </c>
       <c r="D2" t="str">
         <v>Tarek</v>
@@ -507,7 +490,7 @@
         <v>original</v>
       </c>
       <c r="O2" t="str">
-        <v/>
+        <v>ESC-SY-100001</v>
       </c>
     </row>
     <row r="3">
@@ -518,7 +501,7 @@
         <v>Khoury</v>
       </c>
       <c r="C3" t="str">
-        <v/>
+        <v>حنان غسان خوري</v>
       </c>
       <c r="D3" t="str">
         <v>Ghassan</v>
@@ -554,7 +537,7 @@
         <v>associate</v>
       </c>
       <c r="O3" t="str">
-        <v/>
+        <v>ESC-SY-100002</v>
       </c>
     </row>
     <row r="4">
@@ -565,7 +548,7 @@
         <v>Sabbagh</v>
       </c>
       <c r="C4" t="str">
-        <v/>
+        <v>جلال جمال صباغ</v>
       </c>
       <c r="D4" t="str">
         <v>Jamal</v>
@@ -583,7 +566,7 @@
         <v>cardiac_surgery</v>
       </c>
       <c r="I4" t="str">
-        <v/>
+        <v>jalal.sabbagh@scs-net.org</v>
       </c>
       <c r="J4" t="str">
         <v>09931540944</v>
@@ -612,7 +595,7 @@
         <v>Othman</v>
       </c>
       <c r="C5" t="str">
-        <v/>
+        <v>رامي غسان عثمان</v>
       </c>
       <c r="D5" t="str">
         <v>Ghassan</v>
@@ -659,7 +642,7 @@
         <v>Saadeh</v>
       </c>
       <c r="C6" t="str">
-        <v/>
+        <v>لينا يوسف سعادة</v>
       </c>
       <c r="D6" t="str">
         <v>Yousef</v>
@@ -706,7 +689,7 @@
         <v>Mardam-Bey</v>
       </c>
       <c r="C7" t="str">
-        <v/>
+        <v>عدنان غسان مردم بك</v>
       </c>
       <c r="D7" t="str">
         <v>Ghassan</v>
@@ -753,7 +736,7 @@
         <v>Issa</v>
       </c>
       <c r="C8" t="str">
-        <v/>
+        <v>ناجي وليد عيسى</v>
       </c>
       <c r="D8" t="str">
         <v>Walid</v>
@@ -800,7 +783,7 @@
         <v>Mardam-Bey</v>
       </c>
       <c r="C9" t="str">
-        <v/>
+        <v>طارق عدنان مردم بك</v>
       </c>
       <c r="D9" t="str">
         <v>Adnan</v>
@@ -818,7 +801,7 @@
         <v>cardiology</v>
       </c>
       <c r="I9" t="str">
-        <v/>
+        <v>tarek.mardambey@scs-net.org</v>
       </c>
       <c r="J9" t="str">
         <v>09937638166</v>
@@ -847,7 +830,7 @@
         <v>Yacoub</v>
       </c>
       <c r="C10" t="str">
-        <v/>
+        <v>إبراهيم خالد يعقوب</v>
       </c>
       <c r="D10" t="str">
         <v>Khaled</v>
@@ -894,7 +877,7 @@
         <v>Sayegh</v>
       </c>
       <c r="C11" t="str">
-        <v/>
+        <v>مجد طارق صائغ</v>
       </c>
       <c r="D11" t="str">
         <v>Tarek</v>
@@ -930,7 +913,7 @@
         <v>associate</v>
       </c>
       <c r="O11" t="str">
-        <v/>
+        <v>ESC-SY-100010</v>
       </c>
     </row>
     <row r="12">
@@ -941,7 +924,7 @@
         <v>Najjar</v>
       </c>
       <c r="C12" t="str">
-        <v/>
+        <v>بلال علي نجار</v>
       </c>
       <c r="D12" t="str">
         <v>Ali</v>
@@ -977,7 +960,7 @@
         <v>associate</v>
       </c>
       <c r="O12" t="str">
-        <v/>
+        <v>ESC-SY-100011</v>
       </c>
     </row>
     <row r="13">
@@ -988,7 +971,7 @@
         <v>Khoja</v>
       </c>
       <c r="C13" t="str">
-        <v/>
+        <v>يوسف محمود خوجة</v>
       </c>
       <c r="D13" t="str">
         <v>Mahmoud</v>
@@ -1035,7 +1018,7 @@
         <v>Al-Tartousi</v>
       </c>
       <c r="C14" t="str">
-        <v/>
+        <v>صالح وليد الطرطوسي</v>
       </c>
       <c r="D14" t="str">
         <v>Walid</v>
@@ -1071,7 +1054,7 @@
         <v>original</v>
       </c>
       <c r="O14" t="str">
-        <v/>
+        <v>ESC-SY-100013</v>
       </c>
     </row>
     <row r="15">
@@ -1082,7 +1065,7 @@
         <v>Saleh</v>
       </c>
       <c r="C15" t="str">
-        <v/>
+        <v>سامي سامي صالح</v>
       </c>
       <c r="D15" t="str">
         <v>Sami</v>
@@ -1118,7 +1101,7 @@
         <v>original</v>
       </c>
       <c r="O15" t="str">
-        <v/>
+        <v>ESC-SY-100014</v>
       </c>
     </row>
     <row r="16">
@@ -1129,7 +1112,7 @@
         <v>Habib</v>
       </c>
       <c r="C16" t="str">
-        <v/>
+        <v>فارس وليد حبيب</v>
       </c>
       <c r="D16" t="str">
         <v>Walid</v>
@@ -1165,7 +1148,7 @@
         <v>associate</v>
       </c>
       <c r="O16" t="str">
-        <v/>
+        <v>ESC-SY-100015</v>
       </c>
     </row>
     <row r="17">
@@ -1176,7 +1159,7 @@
         <v>Al-Khatib</v>
       </c>
       <c r="C17" t="str">
-        <v/>
+        <v>غادة عدنان الخطيب</v>
       </c>
       <c r="D17" t="str">
         <v>Adnan</v>
@@ -1212,7 +1195,7 @@
         <v>original</v>
       </c>
       <c r="O17" t="str">
-        <v/>
+        <v>ESC-SY-100016</v>
       </c>
     </row>
     <row r="18">
@@ -1223,7 +1206,7 @@
         <v>Sayegh</v>
       </c>
       <c r="C18" t="str">
-        <v/>
+        <v>سامي نبيل صائغ</v>
       </c>
       <c r="D18" t="str">
         <v>Nabil</v>
@@ -1241,7 +1224,7 @@
         <v>cardiac_surgery</v>
       </c>
       <c r="I18" t="str">
-        <v/>
+        <v>sami.sayegh@scs-net.org</v>
       </c>
       <c r="J18" t="str">
         <v>09945392214</v>
@@ -1270,7 +1253,7 @@
         <v>Saleh</v>
       </c>
       <c r="C19" t="str">
-        <v/>
+        <v>مروان عمر صالح</v>
       </c>
       <c r="D19" t="str">
         <v>Omar</v>
@@ -1288,7 +1271,7 @@
         <v>cardiology</v>
       </c>
       <c r="I19" t="str">
-        <v/>
+        <v>marwan.saleh@scs-net.org</v>
       </c>
       <c r="J19" t="str">
         <v>09932510460</v>
@@ -1317,7 +1300,7 @@
         <v>Mansour</v>
       </c>
       <c r="C20" t="str">
-        <v/>
+        <v>غادة سامي منصور</v>
       </c>
       <c r="D20" t="str">
         <v>Sami</v>
@@ -1364,7 +1347,7 @@
         <v>Mansour</v>
       </c>
       <c r="C21" t="str">
-        <v/>
+        <v>زياد محمد منصور</v>
       </c>
       <c r="D21" t="str">
         <v>Mohammad</v>
@@ -1400,7 +1383,7 @@
         <v>original</v>
       </c>
       <c r="O21" t="str">
-        <v/>
+        <v>ESC-SY-100020</v>
       </c>
     </row>
     <row r="22">
@@ -1411,7 +1394,7 @@
         <v>Al-Hamwi</v>
       </c>
       <c r="C22" t="str">
-        <v/>
+        <v>مالك علي الحموي</v>
       </c>
       <c r="D22" t="str">
         <v>Ali</v>
@@ -1429,7 +1412,7 @@
         <v>cardiology</v>
       </c>
       <c r="I22" t="str">
-        <v/>
+        <v>malek.alhamwi@scs-net.org</v>
       </c>
       <c r="J22" t="str">
         <v>09933333946</v>
@@ -1447,7 +1430,7 @@
         <v>original</v>
       </c>
       <c r="O22" t="str">
-        <v/>
+        <v>ESC-SY-100021</v>
       </c>
     </row>
     <row r="23">
@@ -1458,7 +1441,7 @@
         <v>Khalil</v>
       </c>
       <c r="C23" t="str">
-        <v/>
+        <v>مالك محمد خليل</v>
       </c>
       <c r="D23" t="str">
         <v>Mohammad</v>
@@ -1494,7 +1477,7 @@
         <v>original</v>
       </c>
       <c r="O23" t="str">
-        <v/>
+        <v>ESC-SY-100022</v>
       </c>
     </row>
     <row r="24">
@@ -1505,7 +1488,7 @@
         <v>Khoja</v>
       </c>
       <c r="C24" t="str">
-        <v/>
+        <v>وفاء عمر خوجة</v>
       </c>
       <c r="D24" t="str">
         <v>Omar</v>
@@ -1523,7 +1506,7 @@
         <v>cardiac_surgery</v>
       </c>
       <c r="I24" t="str">
-        <v/>
+        <v>wafa.khoja@scs-net.org</v>
       </c>
       <c r="J24" t="str">
         <v>09987284117</v>
@@ -1552,7 +1535,7 @@
         <v>Abdo</v>
       </c>
       <c r="C25" t="str">
-        <v/>
+        <v>سعاد وائل عبدو</v>
       </c>
       <c r="D25" t="str">
         <v>Wael</v>
@@ -1599,7 +1582,7 @@
         <v>Al-Idlibi</v>
       </c>
       <c r="C26" t="str">
-        <v/>
+        <v>سلمى محمد الإدلبي</v>
       </c>
       <c r="D26" t="str">
         <v>Mohammad</v>
@@ -1646,7 +1629,7 @@
         <v>Tlass</v>
       </c>
       <c r="C27" t="str">
-        <v/>
+        <v>سامي حسان طلاس</v>
       </c>
       <c r="D27" t="str">
         <v>Hassan</v>
@@ -1682,7 +1665,7 @@
         <v>original</v>
       </c>
       <c r="O27" t="str">
-        <v/>
+        <v>ESC-SY-100026</v>
       </c>
     </row>
     <row r="28">
@@ -1693,7 +1676,7 @@
         <v>Mardini</v>
       </c>
       <c r="C28" t="str">
-        <v/>
+        <v>نور علي مارديني</v>
       </c>
       <c r="D28" t="str">
         <v>Ali</v>
@@ -1729,7 +1712,7 @@
         <v>associate</v>
       </c>
       <c r="O28" t="str">
-        <v/>
+        <v>ESC-SY-100027</v>
       </c>
     </row>
     <row r="29">
@@ -1740,7 +1723,7 @@
         <v>Al-Ahmad</v>
       </c>
       <c r="C29" t="str">
-        <v/>
+        <v>ناجي جمال الأحمد</v>
       </c>
       <c r="D29" t="str">
         <v>Jamal</v>
@@ -1787,7 +1770,7 @@
         <v>Mardini</v>
       </c>
       <c r="C30" t="str">
-        <v/>
+        <v>تامر وائل مارديني</v>
       </c>
       <c r="D30" t="str">
         <v>Wael</v>
@@ -1823,7 +1806,7 @@
         <v>original</v>
       </c>
       <c r="O30" t="str">
-        <v/>
+        <v>ESC-SY-100029</v>
       </c>
     </row>
     <row r="31">
@@ -1834,7 +1817,7 @@
         <v>Younis</v>
       </c>
       <c r="C31" t="str">
-        <v/>
+        <v>سارة خالد يونس</v>
       </c>
       <c r="D31" t="str">
         <v>Khaled</v>
@@ -1870,7 +1853,7 @@
         <v>original</v>
       </c>
       <c r="O31" t="str">
-        <v/>
+        <v>ESC-SY-100030</v>
       </c>
     </row>
     <row r="32">
@@ -1881,7 +1864,7 @@
         <v>Issa</v>
       </c>
       <c r="C32" t="str">
-        <v/>
+        <v>أسامة عدنان عيسى</v>
       </c>
       <c r="D32" t="str">
         <v>Adnan</v>
@@ -1917,7 +1900,7 @@
         <v>original</v>
       </c>
       <c r="O32" t="str">
-        <v/>
+        <v>ESC-SY-100031</v>
       </c>
     </row>
     <row r="33">
@@ -1928,7 +1911,7 @@
         <v>Al-Ahmad</v>
       </c>
       <c r="C33" t="str">
-        <v/>
+        <v>سيف عماد الأحمد</v>
       </c>
       <c r="D33" t="str">
         <v>Imad</v>
@@ -1975,7 +1958,7 @@
         <v>Khalil</v>
       </c>
       <c r="C34" t="str">
-        <v/>
+        <v>مجد غسان خليل</v>
       </c>
       <c r="D34" t="str">
         <v>Ghassan</v>
@@ -2011,7 +1994,7 @@
         <v>original</v>
       </c>
       <c r="O34" t="str">
-        <v/>
+        <v>ESC-SY-100033</v>
       </c>
     </row>
     <row r="35">
@@ -2022,7 +2005,7 @@
         <v>Bakri</v>
       </c>
       <c r="C35" t="str">
-        <v/>
+        <v>فادي حسان بكري</v>
       </c>
       <c r="D35" t="str">
         <v>Hassan</v>
@@ -2058,7 +2041,7 @@
         <v>original</v>
       </c>
       <c r="O35" t="str">
-        <v/>
+        <v>ESC-SY-100034</v>
       </c>
     </row>
     <row r="36">
@@ -2069,7 +2052,7 @@
         <v>Khalil</v>
       </c>
       <c r="C36" t="str">
-        <v/>
+        <v>ربى غسان خليل</v>
       </c>
       <c r="D36" t="str">
         <v>Ghassan</v>
@@ -2116,7 +2099,7 @@
         <v>Hafez</v>
       </c>
       <c r="C37" t="str">
-        <v/>
+        <v>بشرى محمود حافظ</v>
       </c>
       <c r="D37" t="str">
         <v>Mahmoud</v>
@@ -2163,7 +2146,7 @@
         <v>Issa</v>
       </c>
       <c r="C38" t="str">
-        <v/>
+        <v>هدى وائل عيسى</v>
       </c>
       <c r="D38" t="str">
         <v>Wael</v>
@@ -2199,7 +2182,7 @@
         <v>original</v>
       </c>
       <c r="O38" t="str">
-        <v/>
+        <v>ESC-SY-100037</v>
       </c>
     </row>
     <row r="39">
@@ -2210,7 +2193,7 @@
         <v>Al-Dimashqi</v>
       </c>
       <c r="C39" t="str">
-        <v/>
+        <v>عمر أحمد الدمشقي</v>
       </c>
       <c r="D39" t="str">
         <v>Ahmad</v>
@@ -2257,7 +2240,7 @@
         <v>Al-Kuzbari</v>
       </c>
       <c r="C40" t="str">
-        <v/>
+        <v>طارق بسام الكزبري</v>
       </c>
       <c r="D40" t="str">
         <v>Bassam</v>
@@ -2293,7 +2276,7 @@
         <v>associate</v>
       </c>
       <c r="O40" t="str">
-        <v/>
+        <v>ESC-SY-100039</v>
       </c>
     </row>
     <row r="41">
@@ -2304,7 +2287,7 @@
         <v>Najjar</v>
       </c>
       <c r="C41" t="str">
-        <v/>
+        <v>نجوى طارق نجار</v>
       </c>
       <c r="D41" t="str">
         <v>Tarek</v>
@@ -2340,7 +2323,7 @@
         <v>associate</v>
       </c>
       <c r="O41" t="str">
-        <v/>
+        <v>ESC-SY-100040</v>
       </c>
     </row>
     <row r="42">
@@ -2351,7 +2334,7 @@
         <v>Tabbara</v>
       </c>
       <c r="C42" t="str">
-        <v/>
+        <v>خديجة سامي طبارة</v>
       </c>
       <c r="D42" t="str">
         <v>Sami</v>
@@ -2398,7 +2381,7 @@
         <v>Al-Halabi</v>
       </c>
       <c r="C43" t="str">
-        <v/>
+        <v>فادي نبيل الحلبي</v>
       </c>
       <c r="D43" t="str">
         <v>Nabil</v>
@@ -2434,7 +2417,7 @@
         <v>original</v>
       </c>
       <c r="O43" t="str">
-        <v/>
+        <v>ESC-SY-100042</v>
       </c>
     </row>
     <row r="44">
@@ -2445,7 +2428,7 @@
         <v>Khalil</v>
       </c>
       <c r="C44" t="str">
-        <v/>
+        <v>أحمد عماد خليل</v>
       </c>
       <c r="D44" t="str">
         <v>Imad</v>
@@ -2481,7 +2464,7 @@
         <v>associate</v>
       </c>
       <c r="O44" t="str">
-        <v/>
+        <v>ESC-SY-100043</v>
       </c>
     </row>
     <row r="45">
@@ -2492,7 +2475,7 @@
         <v>Younis</v>
       </c>
       <c r="C45" t="str">
-        <v/>
+        <v>رنا إبراهيم يونس</v>
       </c>
       <c r="D45" t="str">
         <v>Ibrahim</v>
@@ -2510,7 +2493,7 @@
         <v>cardiac_surgery</v>
       </c>
       <c r="I45" t="str">
-        <v/>
+        <v>rana.younis@scs-net.org</v>
       </c>
       <c r="J45" t="str">
         <v>09995510399</v>
@@ -2528,7 +2511,7 @@
         <v>associate</v>
       </c>
       <c r="O45" t="str">
-        <v/>
+        <v>ESC-SY-100044</v>
       </c>
     </row>
     <row r="46">
@@ -2539,7 +2522,7 @@
         <v>Tlass</v>
       </c>
       <c r="C46" t="str">
-        <v/>
+        <v>وسيم عمر طلاس</v>
       </c>
       <c r="D46" t="str">
         <v>Omar</v>
@@ -2586,7 +2569,7 @@
         <v>Haddad</v>
       </c>
       <c r="C47" t="str">
-        <v/>
+        <v>محمود يوسف حداد</v>
       </c>
       <c r="D47" t="str">
         <v>Yousef</v>
@@ -2622,7 +2605,7 @@
         <v>original</v>
       </c>
       <c r="O47" t="str">
-        <v/>
+        <v>ESC-SY-100046</v>
       </c>
     </row>
     <row r="48">
@@ -2633,7 +2616,7 @@
         <v>Al-Homsi</v>
       </c>
       <c r="C48" t="str">
-        <v/>
+        <v>رامز عمر الحمصي</v>
       </c>
       <c r="D48" t="str">
         <v>Omar</v>
@@ -2669,7 +2652,7 @@
         <v>original</v>
       </c>
       <c r="O48" t="str">
-        <v/>
+        <v>ESC-SY-100047</v>
       </c>
     </row>
     <row r="49">
@@ -2680,7 +2663,7 @@
         <v>Abdo</v>
       </c>
       <c r="C49" t="str">
-        <v/>
+        <v>بسام جمال عبدو</v>
       </c>
       <c r="D49" t="str">
         <v>Jamal</v>
@@ -2716,7 +2699,7 @@
         <v>original</v>
       </c>
       <c r="O49" t="str">
-        <v/>
+        <v>ESC-SY-100048</v>
       </c>
     </row>
     <row r="50">
@@ -2727,7 +2710,7 @@
         <v>Aboud</v>
       </c>
       <c r="C50" t="str">
-        <v/>
+        <v>أيمن خالد عبود</v>
       </c>
       <c r="D50" t="str">
         <v>Khaled</v>
@@ -2774,7 +2757,7 @@
         <v>Antaki</v>
       </c>
       <c r="C51" t="str">
-        <v/>
+        <v>تامر نبيل أنطاكي</v>
       </c>
       <c r="D51" t="str">
         <v>Nabil</v>
@@ -2821,7 +2804,7 @@
         <v>Yacoub</v>
       </c>
       <c r="C52" t="str">
-        <v/>
+        <v>عمر عمر يعقوب</v>
       </c>
       <c r="D52" t="str">
         <v>Omar</v>
@@ -2857,7 +2840,7 @@
         <v>original</v>
       </c>
       <c r="O52" t="str">
-        <v/>
+        <v>ESC-SY-100051</v>
       </c>
     </row>
     <row r="53">
@@ -2868,7 +2851,7 @@
         <v>Antaki</v>
       </c>
       <c r="C53" t="str">
-        <v/>
+        <v>سمير سامي أنطاكي</v>
       </c>
       <c r="D53" t="str">
         <v>Sami</v>
@@ -2904,7 +2887,7 @@
         <v>original</v>
       </c>
       <c r="O53" t="str">
-        <v/>
+        <v>ESC-SY-100052</v>
       </c>
     </row>
     <row r="54">
@@ -2915,7 +2898,7 @@
         <v>Al-Halabi</v>
       </c>
       <c r="C54" t="str">
-        <v/>
+        <v>حسان عدنان الحلبي</v>
       </c>
       <c r="D54" t="str">
         <v>Adnan</v>
@@ -2951,7 +2934,7 @@
         <v>associate</v>
       </c>
       <c r="O54" t="str">
-        <v/>
+        <v>ESC-SY-100053</v>
       </c>
     </row>
     <row r="55">
@@ -2962,7 +2945,7 @@
         <v>Al-Idlibi</v>
       </c>
       <c r="C55" t="str">
-        <v/>
+        <v>رامز إبراهيم الإدلبي</v>
       </c>
       <c r="D55" t="str">
         <v>Ibrahim</v>
@@ -3009,7 +2992,7 @@
         <v>Naser</v>
       </c>
       <c r="C56" t="str">
-        <v/>
+        <v>حسين عدنان ناصر</v>
       </c>
       <c r="D56" t="str">
         <v>Adnan</v>
@@ -3056,7 +3039,7 @@
         <v>Al-Kurdi</v>
       </c>
       <c r="C57" t="str">
-        <v/>
+        <v>فيصل جمال الكردي</v>
       </c>
       <c r="D57" t="str">
         <v>Jamal</v>
@@ -3092,7 +3075,7 @@
         <v>original</v>
       </c>
       <c r="O57" t="str">
-        <v/>
+        <v>ESC-SY-100056</v>
       </c>
     </row>
     <row r="58">
@@ -3103,7 +3086,7 @@
         <v>Sabbagh</v>
       </c>
       <c r="C58" t="str">
-        <v/>
+        <v>حنان أحمد صباغ</v>
       </c>
       <c r="D58" t="str">
         <v>Ahmad</v>
@@ -3139,7 +3122,7 @@
         <v>original</v>
       </c>
       <c r="O58" t="str">
-        <v/>
+        <v>ESC-SY-100057</v>
       </c>
     </row>
     <row r="59">
@@ -3150,7 +3133,7 @@
         <v>Sabbagh</v>
       </c>
       <c r="C59" t="str">
-        <v/>
+        <v>محمود محمود صباغ</v>
       </c>
       <c r="D59" t="str">
         <v>Mahmoud</v>
@@ -3186,7 +3169,7 @@
         <v>original</v>
       </c>
       <c r="O59" t="str">
-        <v/>
+        <v>ESC-SY-100058</v>
       </c>
     </row>
     <row r="60">
@@ -3197,7 +3180,7 @@
         <v>Khoja</v>
       </c>
       <c r="C60" t="str">
-        <v/>
+        <v>محمود عمر خوجة</v>
       </c>
       <c r="D60" t="str">
         <v>Omar</v>
@@ -3215,7 +3198,7 @@
         <v>cardiology</v>
       </c>
       <c r="I60" t="str">
-        <v/>
+        <v>mahmoud.khoja@scs-net.org</v>
       </c>
       <c r="J60" t="str">
         <v>09947573815</v>
@@ -3233,7 +3216,7 @@
         <v>associate</v>
       </c>
       <c r="O60" t="str">
-        <v/>
+        <v>ESC-SY-100059</v>
       </c>
     </row>
     <row r="61">
@@ -3244,7 +3227,7 @@
         <v>Al-Shami</v>
       </c>
       <c r="C61" t="str">
-        <v/>
+        <v>خديجة عمر الشامي</v>
       </c>
       <c r="D61" t="str">
         <v>Omar</v>
@@ -3280,7 +3263,7 @@
         <v>original</v>
       </c>
       <c r="O61" t="str">
-        <v/>
+        <v>ESC-SY-100060</v>
       </c>
     </row>
     <row r="62">
@@ -3291,7 +3274,7 @@
         <v>Daouk</v>
       </c>
       <c r="C62" t="str">
-        <v/>
+        <v>وليد غسان داعوق</v>
       </c>
       <c r="D62" t="str">
         <v>Ghassan</v>
@@ -3327,7 +3310,7 @@
         <v>associate</v>
       </c>
       <c r="O62" t="str">
-        <v/>
+        <v>ESC-SY-100061</v>
       </c>
     </row>
     <row r="63">
@@ -3338,7 +3321,7 @@
         <v>Mardam-Bey</v>
       </c>
       <c r="C63" t="str">
-        <v/>
+        <v>كمال عدنان مردم بك</v>
       </c>
       <c r="D63" t="str">
         <v>Adnan</v>
@@ -3385,7 +3368,7 @@
         <v>Bani-Marjeh</v>
       </c>
       <c r="C64" t="str">
-        <v/>
+        <v>محمد عماد بني المرجة</v>
       </c>
       <c r="D64" t="str">
         <v>Imad</v>
@@ -3403,7 +3386,7 @@
         <v>cardiology</v>
       </c>
       <c r="I64" t="str">
-        <v/>
+        <v>mohammad.banimarjeh@scs-net.org</v>
       </c>
       <c r="J64" t="str">
         <v>09944539672</v>
@@ -3421,7 +3404,7 @@
         <v>original</v>
       </c>
       <c r="O64" t="str">
-        <v/>
+        <v>ESC-SY-100063</v>
       </c>
     </row>
     <row r="65">
@@ -3432,7 +3415,7 @@
         <v>Othman</v>
       </c>
       <c r="C65" t="str">
-        <v/>
+        <v>طلال إبراهيم عثمان</v>
       </c>
       <c r="D65" t="str">
         <v>Ibrahim</v>
@@ -3479,7 +3462,7 @@
         <v>Othman</v>
       </c>
       <c r="C66" t="str">
-        <v/>
+        <v>محمد طارق عثمان</v>
       </c>
       <c r="D66" t="str">
         <v>Tarek</v>
@@ -3526,7 +3509,7 @@
         <v>Hafez</v>
       </c>
       <c r="C67" t="str">
-        <v/>
+        <v>بسام وائل حافظ</v>
       </c>
       <c r="D67" t="str">
         <v>Wael</v>
@@ -3573,7 +3556,7 @@
         <v>Issa</v>
       </c>
       <c r="C68" t="str">
-        <v/>
+        <v>وليد محمود عيسى</v>
       </c>
       <c r="D68" t="str">
         <v>Mahmoud</v>
@@ -3609,7 +3592,7 @@
         <v>associate</v>
       </c>
       <c r="O68" t="str">
-        <v/>
+        <v>ESC-SY-100067</v>
       </c>
     </row>
     <row r="69">
@@ -3620,7 +3603,7 @@
         <v>Saleh</v>
       </c>
       <c r="C69" t="str">
-        <v/>
+        <v>إياد وليد صالح</v>
       </c>
       <c r="D69" t="str">
         <v>Walid</v>
@@ -3667,7 +3650,7 @@
         <v>Wakim</v>
       </c>
       <c r="C70" t="str">
-        <v/>
+        <v>تامر إبراهيم وكيم</v>
       </c>
       <c r="D70" t="str">
         <v>Ibrahim</v>
@@ -3703,7 +3686,7 @@
         <v>original</v>
       </c>
       <c r="O70" t="str">
-        <v/>
+        <v>ESC-SY-100069</v>
       </c>
     </row>
     <row r="71">
@@ -3714,7 +3697,7 @@
         <v>Hafez</v>
       </c>
       <c r="C71" t="str">
-        <v/>
+        <v>كمال سامي حافظ</v>
       </c>
       <c r="D71" t="str">
         <v>Sami</v>
@@ -3732,7 +3715,7 @@
         <v>cardiology</v>
       </c>
       <c r="I71" t="str">
-        <v/>
+        <v>kamal.hafez@scs-net.org</v>
       </c>
       <c r="J71" t="str">
         <v>09930401969</v>
@@ -3761,7 +3744,7 @@
         <v>Al-Ahmad</v>
       </c>
       <c r="C72" t="str">
-        <v/>
+        <v>ريم محمد الأحمد</v>
       </c>
       <c r="D72" t="str">
         <v>Mohammad</v>
@@ -3797,7 +3780,7 @@
         <v>original</v>
       </c>
       <c r="O72" t="str">
-        <v/>
+        <v>ESC-SY-100071</v>
       </c>
     </row>
     <row r="73">
@@ -3808,7 +3791,7 @@
         <v>Al-Hassan</v>
       </c>
       <c r="C73" t="str">
-        <v/>
+        <v>صالح حسان الحسن</v>
       </c>
       <c r="D73" t="str">
         <v>Hassan</v>
@@ -3855,7 +3838,7 @@
         <v>Tabbara</v>
       </c>
       <c r="C74" t="str">
-        <v/>
+        <v>سيف طارق طبارة</v>
       </c>
       <c r="D74" t="str">
         <v>Tarek</v>
@@ -3891,7 +3874,7 @@
         <v>associate</v>
       </c>
       <c r="O74" t="str">
-        <v/>
+        <v>ESC-SY-100073</v>
       </c>
     </row>
     <row r="75">
@@ -3902,7 +3885,7 @@
         <v>Haddad</v>
       </c>
       <c r="C75" t="str">
-        <v/>
+        <v>كمال وائل حداد</v>
       </c>
       <c r="D75" t="str">
         <v>Wael</v>
@@ -3949,7 +3932,7 @@
         <v>Al-Shami</v>
       </c>
       <c r="C76" t="str">
-        <v/>
+        <v>زياد بسام الشامي</v>
       </c>
       <c r="D76" t="str">
         <v>Bassam</v>
@@ -3985,7 +3968,7 @@
         <v>original</v>
       </c>
       <c r="O76" t="str">
-        <v/>
+        <v>ESC-SY-100075</v>
       </c>
     </row>
     <row r="77">
@@ -3996,7 +3979,7 @@
         <v>Younis</v>
       </c>
       <c r="C77" t="str">
-        <v/>
+        <v>يارا خالد يونس</v>
       </c>
       <c r="D77" t="str">
         <v>Khaled</v>
@@ -4043,7 +4026,7 @@
         <v>Najjar</v>
       </c>
       <c r="C78" t="str">
-        <v/>
+        <v>فارس حسين نجار</v>
       </c>
       <c r="D78" t="str">
         <v>Hussein</v>
@@ -4090,7 +4073,7 @@
         <v>Al-Halabi</v>
       </c>
       <c r="C79" t="str">
-        <v/>
+        <v>مها سامي الحلبي</v>
       </c>
       <c r="D79" t="str">
         <v>Sami</v>
@@ -4137,7 +4120,7 @@
         <v>Issa</v>
       </c>
       <c r="C80" t="str">
-        <v/>
+        <v>أنس بسام عيسى</v>
       </c>
       <c r="D80" t="str">
         <v>Bassam</v>
@@ -4173,7 +4156,7 @@
         <v>associate</v>
       </c>
       <c r="O80" t="str">
-        <v/>
+        <v>ESC-SY-100079</v>
       </c>
     </row>
     <row r="81">
@@ -4184,7 +4167,7 @@
         <v>Al-Tartousi</v>
       </c>
       <c r="C81" t="str">
-        <v/>
+        <v>بلال خالد الطرطوسي</v>
       </c>
       <c r="D81" t="str">
         <v>Khaled</v>
@@ -4220,7 +4203,7 @@
         <v>original</v>
       </c>
       <c r="O81" t="str">
-        <v/>
+        <v>ESC-SY-100080</v>
       </c>
     </row>
     <row r="82">
@@ -4231,7 +4214,7 @@
         <v>Aboud</v>
       </c>
       <c r="C82" t="str">
-        <v/>
+        <v>سعيد حسان عبود</v>
       </c>
       <c r="D82" t="str">
         <v>Hassan</v>
@@ -4267,7 +4250,7 @@
         <v>original</v>
       </c>
       <c r="O82" t="str">
-        <v/>
+        <v>ESC-SY-100081</v>
       </c>
     </row>
     <row r="83">
@@ -4278,7 +4261,7 @@
         <v>Issa</v>
       </c>
       <c r="C83" t="str">
-        <v/>
+        <v>رنا عدنان عيسى</v>
       </c>
       <c r="D83" t="str">
         <v>Adnan</v>
@@ -4314,7 +4297,7 @@
         <v>original</v>
       </c>
       <c r="O83" t="str">
-        <v/>
+        <v>ESC-SY-100082</v>
       </c>
     </row>
     <row r="84">
@@ -4325,7 +4308,7 @@
         <v>Abdo</v>
       </c>
       <c r="C84" t="str">
-        <v/>
+        <v>كريم أحمد عبدو</v>
       </c>
       <c r="D84" t="str">
         <v>Ahmad</v>
@@ -4372,7 +4355,7 @@
         <v>Aboud</v>
       </c>
       <c r="C85" t="str">
-        <v/>
+        <v>فادي وليد عبود</v>
       </c>
       <c r="D85" t="str">
         <v>Walid</v>
@@ -4408,7 +4391,7 @@
         <v>associate</v>
       </c>
       <c r="O85" t="str">
-        <v/>
+        <v>ESC-SY-100084</v>
       </c>
     </row>
     <row r="86">
@@ -4419,7 +4402,7 @@
         <v>Yacoub</v>
       </c>
       <c r="C86" t="str">
-        <v/>
+        <v>أحمد عدنان يعقوب</v>
       </c>
       <c r="D86" t="str">
         <v>Adnan</v>
@@ -4466,7 +4449,7 @@
         <v>Al-Ahmad</v>
       </c>
       <c r="C87" t="str">
-        <v/>
+        <v>رامي جمال الأحمد</v>
       </c>
       <c r="D87" t="str">
         <v>Jamal</v>
@@ -4502,7 +4485,7 @@
         <v>original</v>
       </c>
       <c r="O87" t="str">
-        <v/>
+        <v>ESC-SY-100086</v>
       </c>
     </row>
     <row r="88">
@@ -4513,7 +4496,7 @@
         <v>Al-Kuzbari</v>
       </c>
       <c r="C88" t="str">
-        <v/>
+        <v>بسام حسين الكزبري</v>
       </c>
       <c r="D88" t="str">
         <v>Hussein</v>
@@ -4560,7 +4543,7 @@
         <v>Al-Kuzbari</v>
       </c>
       <c r="C89" t="str">
-        <v/>
+        <v>رنيم وائل الكزبري</v>
       </c>
       <c r="D89" t="str">
         <v>Wael</v>
@@ -4607,7 +4590,7 @@
         <v>Wakim</v>
       </c>
       <c r="C90" t="str">
-        <v/>
+        <v>رنيم أحمد وكيم</v>
       </c>
       <c r="D90" t="str">
         <v>Ahmad</v>
@@ -4643,7 +4626,7 @@
         <v>original</v>
       </c>
       <c r="O90" t="str">
-        <v/>
+        <v>ESC-SY-100089</v>
       </c>
     </row>
     <row r="91">
@@ -4654,7 +4637,7 @@
         <v>Habib</v>
       </c>
       <c r="C91" t="str">
-        <v/>
+        <v>أيمن عمر حبيب</v>
       </c>
       <c r="D91" t="str">
         <v>Omar</v>
@@ -4690,7 +4673,7 @@
         <v>associate</v>
       </c>
       <c r="O91" t="str">
-        <v/>
+        <v>ESC-SY-100090</v>
       </c>
     </row>
     <row r="92">
@@ -4701,7 +4684,7 @@
         <v>Al-Khatib</v>
       </c>
       <c r="C92" t="str">
-        <v/>
+        <v>داليا حسان الخطيب</v>
       </c>
       <c r="D92" t="str">
         <v>Hassan</v>
@@ -4737,7 +4720,7 @@
         <v>original</v>
       </c>
       <c r="O92" t="str">
-        <v/>
+        <v>ESC-SY-100091</v>
       </c>
     </row>
     <row r="93">
@@ -4748,7 +4731,7 @@
         <v>Al-Tartousi</v>
       </c>
       <c r="C93" t="str">
-        <v/>
+        <v>سعاد بسام الطرطوسي</v>
       </c>
       <c r="D93" t="str">
         <v>Bassam</v>
@@ -4784,7 +4767,7 @@
         <v>associate</v>
       </c>
       <c r="O93" t="str">
-        <v/>
+        <v>ESC-SY-100092</v>
       </c>
     </row>
     <row r="94">
@@ -4795,7 +4778,7 @@
         <v>Chalabi</v>
       </c>
       <c r="C94" t="str">
-        <v/>
+        <v>زياد محمد جلبي</v>
       </c>
       <c r="D94" t="str">
         <v>Mohammad</v>
@@ -4831,7 +4814,7 @@
         <v>associate</v>
       </c>
       <c r="O94" t="str">
-        <v/>
+        <v>ESC-SY-100093</v>
       </c>
     </row>
     <row r="95">
@@ -4842,7 +4825,7 @@
         <v>Atassi</v>
       </c>
       <c r="C95" t="str">
-        <v/>
+        <v>حسان حسان أتاسي</v>
       </c>
       <c r="D95" t="str">
         <v>Hassan</v>
@@ -4889,7 +4872,7 @@
         <v>Tlass</v>
       </c>
       <c r="C96" t="str">
-        <v/>
+        <v>ليلى عدنان طلاس</v>
       </c>
       <c r="D96" t="str">
         <v>Adnan</v>
@@ -4936,7 +4919,7 @@
         <v>Khalil</v>
       </c>
       <c r="C97" t="str">
-        <v/>
+        <v>رنا طارق خليل</v>
       </c>
       <c r="D97" t="str">
         <v>Tarek</v>
@@ -4972,7 +4955,7 @@
         <v>original</v>
       </c>
       <c r="O97" t="str">
-        <v/>
+        <v>ESC-SY-100096</v>
       </c>
     </row>
     <row r="98">
@@ -4983,7 +4966,7 @@
         <v>Mansour</v>
       </c>
       <c r="C98" t="str">
-        <v/>
+        <v>رامي غسان منصور</v>
       </c>
       <c r="D98" t="str">
         <v>Ghassan</v>
@@ -5019,7 +5002,7 @@
         <v>associate</v>
       </c>
       <c r="O98" t="str">
-        <v/>
+        <v>ESC-SY-100097</v>
       </c>
     </row>
     <row r="99">
@@ -5030,7 +5013,7 @@
         <v>Al-Ahmad</v>
       </c>
       <c r="C99" t="str">
-        <v/>
+        <v>طلال جمال الأحمد</v>
       </c>
       <c r="D99" t="str">
         <v>Jamal</v>
@@ -5077,7 +5060,7 @@
         <v>Antaki</v>
       </c>
       <c r="C100" t="str">
-        <v/>
+        <v>ريم عماد أنطاكي</v>
       </c>
       <c r="D100" t="str">
         <v>Imad</v>
@@ -5095,7 +5078,7 @@
         <v>cardiology</v>
       </c>
       <c r="I100" t="str">
-        <v/>
+        <v>reem.antaki@scs-net.org</v>
       </c>
       <c r="J100" t="str">
         <v>09932766490</v>
@@ -5124,7 +5107,7 @@
         <v>Mardini</v>
       </c>
       <c r="C101" t="str">
-        <v/>
+        <v>حسان حسان مارديني</v>
       </c>
       <c r="D101" t="str">
         <v>Hassan</v>
@@ -5171,7 +5154,7 @@
         <v>Bani-Marjeh</v>
       </c>
       <c r="C102" t="str">
-        <v/>
+        <v>مجد أحمد بني المرجة</v>
       </c>
       <c r="D102" t="str">
         <v>Ahmad</v>
@@ -5218,7 +5201,7 @@
         <v>Al-Shami</v>
       </c>
       <c r="C103" t="str">
-        <v/>
+        <v>ربيع وائل الشامي</v>
       </c>
       <c r="D103" t="str">
         <v>Wael</v>
@@ -5265,7 +5248,7 @@
         <v>Khalil</v>
       </c>
       <c r="C104" t="str">
-        <v/>
+        <v>رامي محمد خليل</v>
       </c>
       <c r="D104" t="str">
         <v>Mohammad</v>
@@ -5301,7 +5284,7 @@
         <v>associate</v>
       </c>
       <c r="O104" t="str">
-        <v/>
+        <v>ESC-SY-100103</v>
       </c>
     </row>
     <row r="105">
@@ -5312,7 +5295,7 @@
         <v>Al-Ahmad</v>
       </c>
       <c r="C105" t="str">
-        <v/>
+        <v>داليا غسان الأحمد</v>
       </c>
       <c r="D105" t="str">
         <v>Ghassan</v>
@@ -5348,7 +5331,7 @@
         <v>associate</v>
       </c>
       <c r="O105" t="str">
-        <v/>
+        <v>ESC-SY-100104</v>
       </c>
     </row>
     <row r="106">
@@ -5359,7 +5342,7 @@
         <v>Habib</v>
       </c>
       <c r="C106" t="str">
-        <v/>
+        <v>غسان علي حبيب</v>
       </c>
       <c r="D106" t="str">
         <v>Ali</v>
@@ -5395,7 +5378,7 @@
         <v>original</v>
       </c>
       <c r="O106" t="str">
-        <v/>
+        <v>ESC-SY-100105</v>
       </c>
     </row>
     <row r="107">
@@ -5406,7 +5389,7 @@
         <v>Al-Homsi</v>
       </c>
       <c r="C107" t="str">
-        <v/>
+        <v>نادر غسان الحمصي</v>
       </c>
       <c r="D107" t="str">
         <v>Ghassan</v>
@@ -5453,7 +5436,7 @@
         <v>Sabbagh</v>
       </c>
       <c r="C108" t="str">
-        <v/>
+        <v>فارس طارق صباغ</v>
       </c>
       <c r="D108" t="str">
         <v>Tarek</v>
@@ -5500,7 +5483,7 @@
         <v>Othman</v>
       </c>
       <c r="C109" t="str">
-        <v/>
+        <v>مالك سامي عثمان</v>
       </c>
       <c r="D109" t="str">
         <v>Sami</v>
@@ -5547,7 +5530,7 @@
         <v>Sabbagh</v>
       </c>
       <c r="C110" t="str">
-        <v/>
+        <v>وفاء وليد صباغ</v>
       </c>
       <c r="D110" t="str">
         <v>Walid</v>
@@ -5594,7 +5577,7 @@
         <v>Bakri</v>
       </c>
       <c r="C111" t="str">
-        <v/>
+        <v>أيمن نبيل بكري</v>
       </c>
       <c r="D111" t="str">
         <v>Nabil</v>
@@ -5641,7 +5624,7 @@
         <v>Khoury</v>
       </c>
       <c r="C112" t="str">
-        <v/>
+        <v>سمير جمال خوري</v>
       </c>
       <c r="D112" t="str">
         <v>Jamal</v>
@@ -5688,7 +5671,7 @@
         <v>Saleh</v>
       </c>
       <c r="C113" t="str">
-        <v/>
+        <v>طارق علي صالح</v>
       </c>
       <c r="D113" t="str">
         <v>Ali</v>
@@ -5724,7 +5707,7 @@
         <v>original</v>
       </c>
       <c r="O113" t="str">
-        <v/>
+        <v>ESC-SY-100112</v>
       </c>
     </row>
     <row r="114">
@@ -5735,7 +5718,7 @@
         <v>Tlass</v>
       </c>
       <c r="C114" t="str">
-        <v/>
+        <v>نبيل إبراهيم طلاس</v>
       </c>
       <c r="D114" t="str">
         <v>Ibrahim</v>
@@ -5782,7 +5765,7 @@
         <v>Younis</v>
       </c>
       <c r="C115" t="str">
-        <v/>
+        <v>إياد محمود يونس</v>
       </c>
       <c r="D115" t="str">
         <v>Mahmoud</v>
@@ -5829,7 +5812,7 @@
         <v>Saadeh</v>
       </c>
       <c r="C116" t="str">
-        <v/>
+        <v>نجوى علي سعادة</v>
       </c>
       <c r="D116" t="str">
         <v>Ali</v>
@@ -5876,7 +5859,7 @@
         <v>Haddad</v>
       </c>
       <c r="C117" t="str">
-        <v/>
+        <v>عدنان خالد حداد</v>
       </c>
       <c r="D117" t="str">
         <v>Khaled</v>
@@ -5912,7 +5895,7 @@
         <v>original</v>
       </c>
       <c r="O117" t="str">
-        <v/>
+        <v>ESC-SY-100116</v>
       </c>
     </row>
     <row r="118">
@@ -5923,7 +5906,7 @@
         <v>Al-Homsi</v>
       </c>
       <c r="C118" t="str">
-        <v/>
+        <v>عماد خالد الحمصي</v>
       </c>
       <c r="D118" t="str">
         <v>Khaled</v>
@@ -5959,7 +5942,7 @@
         <v>original</v>
       </c>
       <c r="O118" t="str">
-        <v/>
+        <v>ESC-SY-100117</v>
       </c>
     </row>
     <row r="119">
@@ -5970,7 +5953,7 @@
         <v>Khoja</v>
       </c>
       <c r="C119" t="str">
-        <v/>
+        <v>أسامة بسام خوجة</v>
       </c>
       <c r="D119" t="str">
         <v>Bassam</v>
@@ -6006,7 +5989,7 @@
         <v>associate</v>
       </c>
       <c r="O119" t="str">
-        <v/>
+        <v>ESC-SY-100118</v>
       </c>
     </row>
     <row r="120">
@@ -6017,7 +6000,7 @@
         <v>Al-Idlibi</v>
       </c>
       <c r="C120" t="str">
-        <v/>
+        <v>غسان عماد الإدلبي</v>
       </c>
       <c r="D120" t="str">
         <v>Imad</v>
@@ -6064,7 +6047,7 @@
         <v>Khoury</v>
       </c>
       <c r="C121" t="str">
-        <v/>
+        <v>عدنان طارق خوري</v>
       </c>
       <c r="D121" t="str">
         <v>Tarek</v>
@@ -6100,7 +6083,7 @@
         <v>original</v>
       </c>
       <c r="O121" t="str">
-        <v/>
+        <v>ESC-SY-100120</v>
       </c>
     </row>
     <row r="122">
@@ -6111,7 +6094,7 @@
         <v>Daouk</v>
       </c>
       <c r="C122" t="str">
-        <v/>
+        <v>بشار عمر داعوق</v>
       </c>
       <c r="D122" t="str">
         <v>Omar</v>
@@ -6147,7 +6130,7 @@
         <v>associate</v>
       </c>
       <c r="O122" t="str">
-        <v/>
+        <v>ESC-SY-100121</v>
       </c>
     </row>
     <row r="123">
@@ -6158,7 +6141,7 @@
         <v>Antaki</v>
       </c>
       <c r="C123" t="str">
-        <v/>
+        <v>نادر علي أنطاكي</v>
       </c>
       <c r="D123" t="str">
         <v>Ali</v>
@@ -6194,7 +6177,7 @@
         <v>original</v>
       </c>
       <c r="O123" t="str">
-        <v/>
+        <v>ESC-SY-100122</v>
       </c>
     </row>
     <row r="124">
@@ -6205,7 +6188,7 @@
         <v>Al-Kurdi</v>
       </c>
       <c r="C124" t="str">
-        <v/>
+        <v>علي خالد الكردي</v>
       </c>
       <c r="D124" t="str">
         <v>Khaled</v>
@@ -6223,7 +6206,7 @@
         <v>cardiology</v>
       </c>
       <c r="I124" t="str">
-        <v/>
+        <v>ali.alkurdi@scs-net.org</v>
       </c>
       <c r="J124" t="str">
         <v>09933659597</v>
@@ -6252,7 +6235,7 @@
         <v>Aboud</v>
       </c>
       <c r="C125" t="str">
-        <v/>
+        <v>جلال عماد عبود</v>
       </c>
       <c r="D125" t="str">
         <v>Imad</v>
@@ -6288,7 +6271,7 @@
         <v>associate</v>
       </c>
       <c r="O125" t="str">
-        <v/>
+        <v>ESC-SY-100124</v>
       </c>
     </row>
     <row r="126">
@@ -6299,7 +6282,7 @@
         <v>Sleiman</v>
       </c>
       <c r="C126" t="str">
-        <v/>
+        <v>وسيم وليد سليمان</v>
       </c>
       <c r="D126" t="str">
         <v>Walid</v>
@@ -6346,7 +6329,7 @@
         <v>Saleh</v>
       </c>
       <c r="C127" t="str">
-        <v/>
+        <v>خالد حسان صالح</v>
       </c>
       <c r="D127" t="str">
         <v>Hassan</v>
@@ -6382,7 +6365,7 @@
         <v>original</v>
       </c>
       <c r="O127" t="str">
-        <v/>
+        <v>ESC-SY-100126</v>
       </c>
     </row>
     <row r="128">
@@ -6393,7 +6376,7 @@
         <v>Kanaan</v>
       </c>
       <c r="C128" t="str">
-        <v/>
+        <v>هشام وليد كنعان</v>
       </c>
       <c r="D128" t="str">
         <v>Walid</v>
@@ -6440,7 +6423,7 @@
         <v>Tlass</v>
       </c>
       <c r="C129" t="str">
-        <v/>
+        <v>لمياء علي طلاس</v>
       </c>
       <c r="D129" t="str">
         <v>Ali</v>
@@ -6458,7 +6441,7 @@
         <v>cardiology</v>
       </c>
       <c r="I129" t="str">
-        <v/>
+        <v>lamia.tlass@scs-net.org</v>
       </c>
       <c r="J129" t="str">
         <v>09936369941</v>
@@ -6476,7 +6459,7 @@
         <v>original</v>
       </c>
       <c r="O129" t="str">
-        <v/>
+        <v>ESC-SY-100128</v>
       </c>
     </row>
     <row r="130">
@@ -6487,7 +6470,7 @@
         <v>Al-Ahmad</v>
       </c>
       <c r="C130" t="str">
-        <v/>
+        <v>خالد سامي الأحمد</v>
       </c>
       <c r="D130" t="str">
         <v>Sami</v>
@@ -6534,7 +6517,7 @@
         <v>Bani-Marjeh</v>
       </c>
       <c r="C131" t="str">
-        <v/>
+        <v>تامر حسين بني المرجة</v>
       </c>
       <c r="D131" t="str">
         <v>Hussein</v>
@@ -6581,7 +6564,7 @@
         <v>Al-Halabi</v>
       </c>
       <c r="C132" t="str">
-        <v/>
+        <v>عمر حسان الحلبي</v>
       </c>
       <c r="D132" t="str">
         <v>Hassan</v>
@@ -6628,7 +6611,7 @@
         <v>Khalil</v>
       </c>
       <c r="C133" t="str">
-        <v/>
+        <v>جهاد جمال خليل</v>
       </c>
       <c r="D133" t="str">
         <v>Jamal</v>
@@ -6664,7 +6647,7 @@
         <v>original</v>
       </c>
       <c r="O133" t="str">
-        <v/>
+        <v>ESC-SY-100132</v>
       </c>
     </row>
     <row r="134">
@@ -6675,7 +6658,7 @@
         <v>Wakim</v>
       </c>
       <c r="C134" t="str">
-        <v/>
+        <v>سامي طارق وكيم</v>
       </c>
       <c r="D134" t="str">
         <v>Tarek</v>
@@ -6722,7 +6705,7 @@
         <v>Khalil</v>
       </c>
       <c r="C135" t="str">
-        <v/>
+        <v>مجد إبراهيم خليل</v>
       </c>
       <c r="D135" t="str">
         <v>Ibrahim</v>
@@ -6769,7 +6752,7 @@
         <v>Al-Rifai</v>
       </c>
       <c r="C136" t="str">
-        <v/>
+        <v>غسان أحمد الرفاعي</v>
       </c>
       <c r="D136" t="str">
         <v>Ahmad</v>
@@ -6805,7 +6788,7 @@
         <v>original</v>
       </c>
       <c r="O136" t="str">
-        <v/>
+        <v>ESC-SY-100135</v>
       </c>
     </row>
     <row r="137">
@@ -6816,7 +6799,7 @@
         <v>Tlass</v>
       </c>
       <c r="C137" t="str">
-        <v/>
+        <v>عدنان بسام طلاس</v>
       </c>
       <c r="D137" t="str">
         <v>Bassam</v>
@@ -6863,7 +6846,7 @@
         <v>Saadeh</v>
       </c>
       <c r="C138" t="str">
-        <v/>
+        <v>رنيم علي سعادة</v>
       </c>
       <c r="D138" t="str">
         <v>Ali</v>
@@ -6899,7 +6882,7 @@
         <v>associate</v>
       </c>
       <c r="O138" t="str">
-        <v/>
+        <v>ESC-SY-100137</v>
       </c>
     </row>
     <row r="139">
@@ -6910,7 +6893,7 @@
         <v>Khoja</v>
       </c>
       <c r="C139" t="str">
-        <v/>
+        <v>سمير عمر خوجة</v>
       </c>
       <c r="D139" t="str">
         <v>Omar</v>
@@ -6946,7 +6929,7 @@
         <v>original</v>
       </c>
       <c r="O139" t="str">
-        <v/>
+        <v>ESC-SY-100138</v>
       </c>
     </row>
     <row r="140">
@@ -6957,7 +6940,7 @@
         <v>Saab</v>
       </c>
       <c r="C140" t="str">
-        <v/>
+        <v>أحمد جمال صعب</v>
       </c>
       <c r="D140" t="str">
         <v>Jamal</v>
@@ -7004,7 +6987,7 @@
         <v>Wakim</v>
       </c>
       <c r="C141" t="str">
-        <v/>
+        <v>ريم وليد وكيم</v>
       </c>
       <c r="D141" t="str">
         <v>Walid</v>
@@ -7040,7 +7023,7 @@
         <v>associate</v>
       </c>
       <c r="O141" t="str">
-        <v/>
+        <v>ESC-SY-100140</v>
       </c>
     </row>
     <row r="142">
@@ -7051,7 +7034,7 @@
         <v>Daouk</v>
       </c>
       <c r="C142" t="str">
-        <v/>
+        <v>جهاد حسان داعوق</v>
       </c>
       <c r="D142" t="str">
         <v>Hassan</v>
@@ -7098,7 +7081,7 @@
         <v>Al-Homsi</v>
       </c>
       <c r="C143" t="str">
-        <v/>
+        <v>بشار نبيل الحمصي</v>
       </c>
       <c r="D143" t="str">
         <v>Nabil</v>
@@ -7134,7 +7117,7 @@
         <v>associate</v>
       </c>
       <c r="O143" t="str">
-        <v/>
+        <v>ESC-SY-100142</v>
       </c>
     </row>
     <row r="144">
@@ -7145,7 +7128,7 @@
         <v>Mansour</v>
       </c>
       <c r="C144" t="str">
-        <v/>
+        <v>محمد طارق منصور</v>
       </c>
       <c r="D144" t="str">
         <v>Tarek</v>
@@ -7163,7 +7146,7 @@
         <v>cardiology</v>
       </c>
       <c r="I144" t="str">
-        <v/>
+        <v>mohammad.mansour@scs-net.org</v>
       </c>
       <c r="J144" t="str">
         <v>09934822210</v>
@@ -7181,7 +7164,7 @@
         <v>original</v>
       </c>
       <c r="O144" t="str">
-        <v/>
+        <v>ESC-SY-100143</v>
       </c>
     </row>
     <row r="145">
@@ -7192,7 +7175,7 @@
         <v>Al-Hassan</v>
       </c>
       <c r="C145" t="str">
-        <v/>
+        <v>فيصل بسام الحسن</v>
       </c>
       <c r="D145" t="str">
         <v>Bassam</v>
@@ -7210,7 +7193,7 @@
         <v>cardiology</v>
       </c>
       <c r="I145" t="str">
-        <v/>
+        <v>faisal.alhassan@scs-net.org</v>
       </c>
       <c r="J145" t="str">
         <v>09991669093</v>
@@ -7239,7 +7222,7 @@
         <v>Saab</v>
       </c>
       <c r="C146" t="str">
-        <v/>
+        <v>يوسف نبيل صعب</v>
       </c>
       <c r="D146" t="str">
         <v>Nabil</v>
@@ -7275,7 +7258,7 @@
         <v>original</v>
       </c>
       <c r="O146" t="str">
-        <v/>
+        <v>ESC-SY-100145</v>
       </c>
     </row>
     <row r="147">
@@ -7286,7 +7269,7 @@
         <v>Khalil</v>
       </c>
       <c r="C147" t="str">
-        <v/>
+        <v>حسان عماد خليل</v>
       </c>
       <c r="D147" t="str">
         <v>Imad</v>
@@ -7322,7 +7305,7 @@
         <v>original</v>
       </c>
       <c r="O147" t="str">
-        <v/>
+        <v>ESC-SY-100146</v>
       </c>
     </row>
     <row r="148">
@@ -7333,7 +7316,7 @@
         <v>Saab</v>
       </c>
       <c r="C148" t="str">
-        <v/>
+        <v>زياد عماد صعب</v>
       </c>
       <c r="D148" t="str">
         <v>Imad</v>
@@ -7380,7 +7363,7 @@
         <v>Othman</v>
       </c>
       <c r="C149" t="str">
-        <v/>
+        <v>حسان طارق عثمان</v>
       </c>
       <c r="D149" t="str">
         <v>Tarek</v>
@@ -7427,7 +7410,7 @@
         <v>Khoja</v>
       </c>
       <c r="C150" t="str">
-        <v/>
+        <v>وسيم محمود خوجة</v>
       </c>
       <c r="D150" t="str">
         <v>Mahmoud</v>
@@ -7474,7 +7457,7 @@
         <v>Al-Rifai</v>
       </c>
       <c r="C151" t="str">
-        <v/>
+        <v>بشار نبيل الرفاعي</v>
       </c>
       <c r="D151" t="str">
         <v>Nabil</v>
@@ -7510,7 +7493,7 @@
         <v>original</v>
       </c>
       <c r="O151" t="str">
-        <v/>
+        <v>ESC-SY-100150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>